<commit_message>
chore: update data exports and anomaly database records
</commit_message>
<xml_diff>
--- a/data/exports/Executive_Retail_Sales_Inventory_Report.xlsx
+++ b/data/exports/Executive_Retail_Sales_Inventory_Report.xlsx
@@ -179,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -211,6 +211,7 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -792,7 +793,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated On: 2026-10-16 09:51 | Multi-Store Performance &amp; 18% Stockout Reduction Scorecard</t>
+          <t>Generated On: 2026-10-16 11:31 | Multi-Store Performance &amp; 18% Stockout Reduction Scorecard</t>
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
@@ -2580,14 +2581,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -2644,6 +2645,1086 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Chicago Michigan Ave Center</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Apparel</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>French Terry Oversized Hoodie</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Demand Surge</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>3.71</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Dallas Galleria Megastore</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Motorized Standing Desk Converter</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Demand Surge</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Seattle Pike Place Boutique</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Apparel</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Lightweight Packable Windbreaker</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Demand Surge</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>3.39</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Omnichannel Hub &amp; Express</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Minimalist Daily Canvas Sneaker</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Demand Surge</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Artisan Compact Espresso Machine</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>HEPA Smart Air Purifier Pro</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Pre-Seasoned Cast Iron Dutch Oven</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Motorized Standing Desk Converter</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Minimalist Ceramic Dinnerware Set 16pc</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Cordless Stick Vacuum Ultra</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Handcrafted Italian Leather Loafers</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H15" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Water-Resistant Winter Snow Boot</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Luxury &amp; Accessories</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Full-Grain Leather Weekender Duffle</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H17" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Luxury &amp; Accessories</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Pure Cashmere Fringed Scarf</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H18" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Manhattan 5th Ave Flagship</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Luxury &amp; Accessories</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Handcrafted Brass Desk Clock</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H19" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chicago Michigan Ave Center</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Artisan Compact Espresso Machine</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H20" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Chicago Michigan Ave Center</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Motorized Standing Desk Converter</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H21" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Chicago Michigan Ave Center</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Cordless Stick Vacuum Ultra</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H22" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Chicago Michigan Ave Center</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Handcrafted Italian Leather Loafers</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H23" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Artisan Compact Espresso Machine</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>HEPA Smart Air Purifier Pro</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H25" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Pre-Seasoned Cast Iron Dutch Oven</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Minimalist Ceramic Dinnerware Set 16pc</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Home &amp; Living</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Cordless Stick Vacuum Ultra</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H28" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>All-Weather Waterproof Trail Boot</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H29" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Goodyear Welted Suede Chelsea Boot</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Footwear</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Water-Resistant Winter Snow Boot</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H31" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Luxury &amp; Accessories</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Full-Grain Leather Weekender Duffle</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>SF Union Square Tech Hub</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Luxury &amp; Accessories</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Pure Cashmere Fringed Scarf</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H33" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Austin Domain Town Center</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Apparel</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Waterproof Thermal Mountain Parka</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Stockout Event</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>-3.2</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H2"/>

</xml_diff>